<commit_message>
create Clock and Bewerbs-Structure
</commit_message>
<xml_diff>
--- a/additional Files/web-with-googlesheet_260501-1015.xlsx
+++ b/additional Files/web-with-googlesheet_260501-1015.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\pro\GitHub\GitHub\WebApp-with-GoogleSheet_comunication\additional Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{744CC62D-2024-4C82-914E-7605D4B8B714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D931CAB-9D6C-4C27-BD29-FA67F7803927}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Personen" sheetId="1" r:id="rId1"/>
@@ -356,9 +356,6 @@
     <t>Einfaches gewertetes Spiel</t>
   </si>
   <si>
-    <t>Rangliste</t>
-  </si>
-  <si>
     <t>Rasterkonfiguration 16</t>
   </si>
   <si>
@@ -383,9 +380,6 @@
     <t>Gewerteter Einzelvergleichskamp</t>
   </si>
   <si>
-    <t>Beispiel Rangliste</t>
-  </si>
-  <si>
     <t>Rangliste Damen</t>
   </si>
   <si>
@@ -399,6 +393,12 @@
   </si>
   <si>
     <t>Entrydate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rangliste </t>
+  </si>
+  <si>
+    <t>Rangliste Herren</t>
   </si>
 </sst>
 </file>
@@ -410,7 +410,7 @@
     <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -448,6 +448,13 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -457,7 +464,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -465,11 +472,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -499,6 +521,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -786,7 +814,7 @@
       <c r="Y1" s="3"/>
       <c r="Z1" s="3"/>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -807,7 +835,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -821,7 +849,7 @@
       <c r="F3" s="4"/>
       <c r="J3" s="4"/>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -835,7 +863,7 @@
       <c r="F4" s="4"/>
       <c r="J4" s="4"/>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -849,7 +877,7 @@
       <c r="F5" s="4"/>
       <c r="J5" s="4"/>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -863,7 +891,7 @@
       <c r="F6" s="4"/>
       <c r="J6" s="4"/>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -877,7 +905,7 @@
       <c r="F7" s="4"/>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -891,7 +919,7 @@
       <c r="F8" s="4"/>
       <c r="J8" s="4"/>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -905,7 +933,7 @@
       <c r="F9" s="4"/>
       <c r="J9" s="4"/>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -919,7 +947,7 @@
       <c r="F10" s="4"/>
       <c r="J10" s="4"/>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -937,7 +965,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -951,7 +979,7 @@
       <c r="F12" s="4"/>
       <c r="J12" s="4"/>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -965,7 +993,7 @@
       <c r="F13" s="4"/>
       <c r="J13" s="4"/>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -983,7 +1011,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A15" s="4">
         <v>14</v>
       </c>
@@ -1001,7 +1029,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -1019,7 +1047,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A17" s="4">
         <v>16</v>
       </c>
@@ -1037,7 +1065,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A18" s="4">
         <v>17</v>
       </c>
@@ -1055,7 +1083,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A19" s="4">
         <v>18</v>
       </c>
@@ -1073,7 +1101,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A20" s="4">
         <v>19</v>
       </c>
@@ -1091,7 +1119,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A21" s="4"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -1099,7 +1127,7 @@
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A22" s="4"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -1107,7 +1135,7 @@
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A23" s="4"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -1115,7 +1143,7 @@
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A24" s="4"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -1123,7 +1151,7 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A25" s="4"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -1131,7 +1159,7 @@
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A26" s="4"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -1139,7 +1167,7 @@
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A27" s="4"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -1147,7 +1175,7 @@
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -1155,7 +1183,7 @@
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -1163,7 +1191,7 @@
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A30" s="4"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -1171,7 +1199,7 @@
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A31" s="4"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -1179,7 +1207,7 @@
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A32" s="4"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -1187,7 +1215,7 @@
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A33" s="4"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -1195,7 +1223,7 @@
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A34" s="4"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -1203,7 +1231,7 @@
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A35" s="4"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -1211,7 +1239,7 @@
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A36" s="4"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -1219,7 +1247,7 @@
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A37" s="4"/>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -1227,7 +1255,7 @@
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A38" s="4"/>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
@@ -1235,7 +1263,7 @@
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A39" s="4"/>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
@@ -1243,7 +1271,7 @@
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A40" s="4"/>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -1251,7 +1279,7 @@
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A41" s="4"/>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -1259,7 +1287,7 @@
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A42" s="4"/>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -8952,186 +8980,201 @@
   <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="14" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2">
+    <row r="2" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="15">
         <v>2</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="15">
         <v>1</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="15">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3">
+      <c r="D2" s="14"/>
+    </row>
+    <row r="3" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="15">
         <v>2</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="15">
         <v>2</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="15">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4">
+      <c r="D3" s="14"/>
+    </row>
+    <row r="4" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="15">
         <v>2</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="15">
         <v>3</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="15">
+        <v>15</v>
+      </c>
+      <c r="D4" s="14"/>
+    </row>
+    <row r="5" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="15">
+        <v>2</v>
+      </c>
+      <c r="B5" s="15">
+        <v>4</v>
+      </c>
+      <c r="C5" s="15">
+        <v>4</v>
+      </c>
+      <c r="D5" s="14"/>
+    </row>
+    <row r="6" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="15">
+        <v>2</v>
+      </c>
+      <c r="B6" s="15">
+        <v>5</v>
+      </c>
+      <c r="C6" s="15">
+        <v>6</v>
+      </c>
+      <c r="D6" s="14"/>
+    </row>
+    <row r="7" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="15">
+        <v>2</v>
+      </c>
+      <c r="B7" s="15">
+        <v>6</v>
+      </c>
+      <c r="C7" s="15">
+        <v>8</v>
+      </c>
+      <c r="D7" s="14"/>
+    </row>
+    <row r="8" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="15">
+        <v>2</v>
+      </c>
+      <c r="B8" s="15">
+        <v>7</v>
+      </c>
+      <c r="C8" s="15">
+        <v>2</v>
+      </c>
+      <c r="D8" s="14"/>
+    </row>
+    <row r="9" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="15">
+        <v>2</v>
+      </c>
+      <c r="B9" s="15">
+        <v>8</v>
+      </c>
+      <c r="C9" s="15">
+        <v>7</v>
+      </c>
+      <c r="D9" s="14"/>
+    </row>
+    <row r="10" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="15">
+        <v>2</v>
+      </c>
+      <c r="B10" s="15">
+        <v>9</v>
+      </c>
+      <c r="C10" s="15">
+        <v>9</v>
+      </c>
+      <c r="D10" s="14"/>
+    </row>
+    <row r="11" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="15">
+        <v>2</v>
+      </c>
+      <c r="B11" s="15">
+        <v>10</v>
+      </c>
+      <c r="C11" s="15">
+        <v>14</v>
+      </c>
+      <c r="D11" s="14"/>
+    </row>
+    <row r="12" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="15">
+        <v>2</v>
+      </c>
+      <c r="B12" s="15">
+        <v>11</v>
+      </c>
+      <c r="C12" s="15">
+        <v>1</v>
+      </c>
+      <c r="D12" s="14"/>
+    </row>
+    <row r="13" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="15">
+        <v>3</v>
+      </c>
+      <c r="B13" s="15">
+        <v>1</v>
+      </c>
+      <c r="C13" s="15">
+        <v>11</v>
+      </c>
+      <c r="D13" s="14"/>
+    </row>
+    <row r="14" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="15">
+        <v>3</v>
+      </c>
+      <c r="B14" s="15">
+        <v>2</v>
+      </c>
+      <c r="C14" s="15">
+        <v>12</v>
+      </c>
+      <c r="D14" s="14"/>
+    </row>
+    <row r="15" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="15">
+        <v>3</v>
+      </c>
+      <c r="B15" s="15">
+        <v>3</v>
+      </c>
+      <c r="C15" s="15">
+        <v>3</v>
+      </c>
+      <c r="D15" s="14"/>
+    </row>
+    <row r="16" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="15">
+        <v>3</v>
+      </c>
+      <c r="B16" s="15">
+        <v>4</v>
+      </c>
+      <c r="C16" s="15">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5" s="5">
-        <v>4</v>
-      </c>
-      <c r="C5" s="5">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>2</v>
-      </c>
-      <c r="B6" s="5">
-        <v>5</v>
-      </c>
-      <c r="C6" s="5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>2</v>
-      </c>
-      <c r="B7" s="5">
-        <v>6</v>
-      </c>
-      <c r="C7" s="5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>2</v>
-      </c>
-      <c r="B8" s="5">
-        <v>7</v>
-      </c>
-      <c r="C8" s="5">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>2</v>
-      </c>
-      <c r="B9" s="5">
-        <v>8</v>
-      </c>
-      <c r="C9" s="5">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>2</v>
-      </c>
-      <c r="B10" s="5">
-        <v>9</v>
-      </c>
-      <c r="C10" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>2</v>
-      </c>
-      <c r="B11" s="5">
-        <v>10</v>
-      </c>
-      <c r="C11" s="5">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>2</v>
-      </c>
-      <c r="B12" s="5">
-        <v>11</v>
-      </c>
-      <c r="C12" s="5">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>2</v>
-      </c>
-      <c r="B13" s="5">
-        <v>12</v>
-      </c>
-      <c r="C13" s="5">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14">
-        <v>2</v>
-      </c>
-      <c r="B14" s="5">
-        <v>13</v>
-      </c>
-      <c r="C14" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15">
-        <v>2</v>
-      </c>
-      <c r="B15" s="5">
-        <v>14</v>
-      </c>
-      <c r="C15" s="5">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16">
-        <v>2</v>
-      </c>
-      <c r="B16" s="5">
-        <v>15</v>
-      </c>
-      <c r="C16" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="D16" s="14"/>
+    </row>
+    <row r="17" spans="2:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B17" s="8"/>
     </row>
   </sheetData>
@@ -9801,7 +9844,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="C3" s="13">
         <v>1</v>
@@ -9817,7 +9860,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="13">
@@ -9833,7 +9876,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="13">
@@ -9865,22 +9908,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>90</v>
       </c>
       <c r="D1" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="E1" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="F1" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="G1" s="7" t="s">
         <v>115</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -9891,7 +9934,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D2" s="7"/>
       <c r="E2" s="7"/>
@@ -9906,7 +9949,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -9923,7 +9966,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
@@ -9940,7 +9983,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
@@ -9957,11 +10000,11 @@
         <v>4</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D6" s="7"/>
       <c r="E6" s="7" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F6" s="13">
         <v>20260701</v>
@@ -9989,7 +10032,7 @@
         <v>66</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>